<commit_message>
update show value main
</commit_message>
<xml_diff>
--- a/Plan.xlsx
+++ b/Plan.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\App\Production\Extruder3\Application\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F8D2C2-7E94-488A-812B-3F7BD62380FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2551FA97-6EA4-4864-99BE-7300C2BFF04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED8BDF50-8AB4-4219-88FA-76AB31D70C70}"/>
   </bookViews>
@@ -65,21 +65,66 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>07PB1M2-Xe</t>
+  </si>
+  <si>
+    <t>07PD1M2-Xe</t>
+  </si>
+  <si>
+    <t>07PD2M2-Xe</t>
+  </si>
+  <si>
+    <t>07PE1M2-Xe</t>
+  </si>
+  <si>
+    <t>07PE2M2-Xe</t>
+  </si>
+  <si>
+    <t>07PE3M2-Xe</t>
+  </si>
+  <si>
+    <t>07PE4M2-Xe</t>
+  </si>
   <si>
     <t>06PE1M2-Xe</t>
+  </si>
+  <si>
+    <t>07PD3M2-Xe</t>
   </si>
   <si>
     <t>06PE2M2-Xe</t>
   </si>
   <si>
+    <t>06PE3M2-Xe</t>
+  </si>
+  <si>
     <t>06J51A2-Roll</t>
+  </si>
+  <si>
+    <t>07PB1M3-Xe</t>
+  </si>
+  <si>
+    <t>07PD1M3-Xe</t>
+  </si>
+  <si>
+    <t>07PD2M3-Xe</t>
   </si>
   <si>
     <t>03PE1M3-Xe</t>
   </si>
   <si>
+    <t>07PE1M3-Xe</t>
+  </si>
+  <si>
+    <t>07PE3M3-Xe</t>
+  </si>
+  <si>
     <t>06PE1M3-Xe</t>
+  </si>
+  <si>
+    <t>07PD3M3-Xe</t>
   </si>
   <si>
     <t>06PE1TR3-Xe</t>
@@ -195,9 +240,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -212,6 +254,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -263,10 +308,10 @@
       <sheetName val="Helper"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4">
         <row r="4">
           <cell r="A4">
@@ -3077,7 +3122,7 @@
         </row>
       </sheetData>
       <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="6" refreshError="1"/>
       <sheetData sheetId="7">
         <row r="2">
           <cell r="C2" t="str">
@@ -3219,8 +3264,8 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3600,68 +3645,188 @@
   <sheetPr codeName="Sheet3">
     <tabColor indexed="17"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="24.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" style="6" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="5" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="9.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" style="4" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" ht="54" customHeight="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A2" s="7">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A3" s="7">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A4" s="7">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="7" t="s">
+    </row>
+    <row r="5" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A5" s="7">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A7" s="7">
         <v>6</v>
       </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A2" s="2">
+    <row r="8" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A11" s="7">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A13" s="7">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>2</v>
+    <row r="18" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>0</v>
+    <row r="19" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>4</v>
+    <row r="20" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>5</v>
+    <row r="21" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A21" s="7">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="4" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A7" s="2">
+    <row r="22" spans="1:2" ht="24.75" customHeight="1">
+      <c r="A22" s="7">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update logic import add plan
</commit_message>
<xml_diff>
--- a/Plan.xlsx
+++ b/Plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\App\Production\Extruder3\Application\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2551FA97-6EA4-4864-99BE-7300C2BFF04C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57FFD6D-9E92-41B5-B424-435DE3ADA881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED8BDF50-8AB4-4219-88FA-76AB31D70C70}"/>
   </bookViews>
@@ -31,7 +31,7 @@
     <definedName name="mac">INDEX([1]DataMaster1!#REF!,MATCH('[2]Cuốn roll'!$G$8:$H$8,[1]DataMaster1!$A$4:$A$297,0))</definedName>
     <definedName name="macroll" localSheetId="0">INDEX(DATA!#REF!,MATCH(#REF!,DATA!$A$2:$A$7,0))</definedName>
     <definedName name="macroll">INDEX([1]DataMaster1!#REF!,MATCH('[2]Roll (BIMC)'!$G$7:$H$7,[1]DataMaster1!$A$4:$A$297,0))</definedName>
-    <definedName name="rol" localSheetId="0">INDEX(DATA!#REF!,MATCH(#REF!,DATA!$A$2:$A$144,0))</definedName>
+    <definedName name="rol" localSheetId="0">INDEX(DATA!#REF!,MATCH(#REF!,DATA!$A$2:$A$130,0))</definedName>
     <definedName name="rol">INDEX([1]DataMaster1!#REF!,MATCH('[2]Roll (BIMC)'!$G$7:$H$7,[1]DataMaster1!$A$4:$A$528,0))</definedName>
     <definedName name="roll" localSheetId="0">INDEX(DATA!#REF!,MATCH(#REF!,DATA!$A$2:$A$7,0))</definedName>
     <definedName name="roll">INDEX([1]DataMaster1!#REF!,MATCH('[2]Cuốn roll'!$G$8:$H$8,[1]DataMaster1!$A$4:$A$297,0))</definedName>
@@ -65,66 +65,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>07PB1M2-Xe</t>
-  </si>
-  <si>
-    <t>07PD1M2-Xe</t>
-  </si>
-  <si>
-    <t>07PD2M2-Xe</t>
-  </si>
-  <si>
-    <t>07PE1M2-Xe</t>
-  </si>
-  <si>
-    <t>07PE2M2-Xe</t>
-  </si>
-  <si>
-    <t>07PE3M2-Xe</t>
-  </si>
-  <si>
-    <t>07PE4M2-Xe</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>06PE1M2-Xe</t>
-  </si>
-  <si>
-    <t>07PD3M2-Xe</t>
   </si>
   <si>
     <t>06PE2M2-Xe</t>
   </si>
   <si>
-    <t>06PE3M2-Xe</t>
-  </si>
-  <si>
     <t>06J51A2-Roll</t>
-  </si>
-  <si>
-    <t>07PB1M3-Xe</t>
-  </si>
-  <si>
-    <t>07PD1M3-Xe</t>
   </si>
   <si>
     <t>07PD2M3-Xe</t>
   </si>
   <si>
     <t>03PE1M3-Xe</t>
-  </si>
-  <si>
-    <t>07PE1M3-Xe</t>
-  </si>
-  <si>
-    <t>07PE3M3-Xe</t>
-  </si>
-  <si>
-    <t>06PE1M3-Xe</t>
-  </si>
-  <si>
-    <t>07PD3M3-Xe</t>
   </si>
   <si>
     <t>06PE1TR3-Xe</t>
@@ -134,6 +89,9 @@
   </si>
   <si>
     <t>Stt</t>
+  </si>
+  <si>
+    <t>plan_code</t>
   </si>
 </sst>
 </file>
@@ -265,7 +223,127 @@
     <cellStyle name="Normal 4" xfId="3" xr:uid="{8C7EC361-91D0-47E5-81D0-D94454C4DF8F}"/>
     <cellStyle name="Normal_Sheet1" xfId="2" xr:uid="{114BF478-45E3-450F-BDE7-EE649C429F61}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="13">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3645,195 +3723,309 @@
   <sheetPr codeName="Sheet3">
     <tabColor indexed="17"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="24.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="9.7109375" style="5" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="4"/>
+    <col min="3" max="3" width="26.42578125" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="54" customHeight="1">
+    <row r="1" spans="1:7" s="1" customFormat="1" ht="54" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>21</v>
+        <v>6</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+    <row r="2" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
       <c r="A2" s="7">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>15</v>
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <f ca="1">B2&amp;"_"&amp;ROUND(NOW(),0)&amp;A2</f>
+        <v>03PE1M3-Xe_461721</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+    <row r="3" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
       <c r="A3" s="7">
+        <f>IF(B3&lt;&gt;"",A2+1,"")</f>
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>11</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <f t="shared" ref="C3" ca="1" si="0">B3&amp;"_"&amp;ROUND(NOW(),0)&amp;A3</f>
+        <v>06J51A2-Roll_461722</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
+    <row r="4" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
       <c r="A4" s="7">
+        <f>IF(B4&lt;&gt;"",A3+1,"")</f>
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <f ca="1">B4&amp;"_"&amp;ROUND(NOW(),0)&amp;A4</f>
+        <v>06J51A2-Roll_461723</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A5" s="7">
+        <f>IF(B5&lt;&gt;"",A4+1,"")</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <f ca="1">B5&amp;"_"&amp;ROUND(NOW(),0)&amp;A5</f>
+        <v>06PE1M2-Xe_461724</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A6" s="7">
+        <f>IF(B6&lt;&gt;"",A5+1,"")</f>
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <f ca="1">B6&amp;"_"&amp;ROUND(NOW(),0)&amp;A6</f>
+        <v>06PE1TR3-Xe_461725</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="3" customFormat="1" ht="24.75" customHeight="1">
+      <c r="A7" s="7">
+        <f>IF(B7&lt;&gt;"",A6+1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <f ca="1">B7&amp;"_"&amp;ROUND(NOW(),0)&amp;A7</f>
+        <v>06PE2M2-Xe_461726</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A8" s="7">
+        <f>IF(B8&lt;&gt;"",A7+1,"")</f>
         <v>7</v>
       </c>
+      <c r="B8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <f ca="1">IF(B8&lt;&gt;"",B8&amp;"_"&amp;ROUND(NOW(),0)&amp;A8,"")</f>
+        <v>07PD2M3-Xe_461727</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A5" s="7">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>18</v>
+    <row r="9" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A9" s="7">
+        <f>IF(B9&lt;&gt;"",A8+1,"")</f>
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <f ca="1">IF(B9&lt;&gt;"",B9&amp;"_"&amp;ROUND(NOW(),0)&amp;A9,"")</f>
+        <v>07PD2M3-Xe_461728</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A6" s="7">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
+    <row r="10" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A10" s="7" t="str">
+        <f>IF(B10&lt;&gt;"",A9+1,"")</f>
+        <v/>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2" t="str">
+        <f ca="1">IF(B10&lt;&gt;"",B10&amp;"_"&amp;ROUND(NOW(),0)&amp;A10,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="7" spans="1:2" s="3" customFormat="1" ht="24.75" customHeight="1">
-      <c r="A7" s="7">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
+    <row r="11" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A11" s="7" t="str">
+        <f>IF(B11&lt;&gt;"",A10+1,"")</f>
+        <v/>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="str">
+        <f ca="1">IF(B11&lt;&gt;"",B11&amp;"_"&amp;ROUND(NOW(),0)&amp;A11,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A8" s="7">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>10</v>
+    <row r="12" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A12" s="7" t="str">
+        <f>IF(B12&lt;&gt;"",A11+1,"")</f>
+        <v/>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="str">
+        <f ca="1">IF(B12&lt;&gt;"",B12&amp;"_"&amp;ROUND(NOW(),0)&amp;A12,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A9" s="7">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>0</v>
+    <row r="13" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A13" s="7" t="str">
+        <f>IF(B13&lt;&gt;"",A12+1,"")</f>
+        <v/>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2" t="str">
+        <f ca="1">IF(B13&lt;&gt;"",B13&amp;"_"&amp;ROUND(NOW(),0)&amp;A13,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A10" s="7">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>12</v>
+    <row r="14" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A14" s="7" t="str">
+        <f>IF(B14&lt;&gt;"",A13+1,"")</f>
+        <v/>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="str">
+        <f ca="1">IF(B14&lt;&gt;"",B14&amp;"_"&amp;ROUND(NOW(),0)&amp;A14,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A11" s="7">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>1</v>
+    <row r="15" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A15" s="7" t="str">
+        <f>IF(B15&lt;&gt;"",A14+1,"")</f>
+        <v/>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="str">
+        <f ca="1">IF(B15&lt;&gt;"",B15&amp;"_"&amp;ROUND(NOW(),0)&amp;A15,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A12" s="7">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>13</v>
+    <row r="16" spans="1:7" ht="24.75" customHeight="1">
+      <c r="A16" s="7" t="str">
+        <f>IF(B16&lt;&gt;"",A15+1,"")</f>
+        <v/>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="str">
+        <f ca="1">IF(B16&lt;&gt;"",B16&amp;"_"&amp;ROUND(NOW(),0)&amp;A16,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A13" s="7">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>2</v>
+    <row r="17" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A17" s="7" t="str">
+        <f>IF(B17&lt;&gt;"",A16+1,"")</f>
+        <v/>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2" t="str">
+        <f ca="1">IF(B17&lt;&gt;"",B17&amp;"_"&amp;ROUND(NOW(),0)&amp;A17,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A14" s="7">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>14</v>
+    <row r="18" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A18" s="7" t="str">
+        <f>IF(B18&lt;&gt;"",A17+1,"")</f>
+        <v/>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2" t="str">
+        <f ca="1">IF(B18&lt;&gt;"",B18&amp;"_"&amp;ROUND(NOW(),0)&amp;A18,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A15" s="7">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>8</v>
+    <row r="19" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A19" s="7" t="str">
+        <f>IF(B19&lt;&gt;"",A18+1,"")</f>
+        <v/>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2" t="str">
+        <f ca="1">IF(B19&lt;&gt;"",B19&amp;"_"&amp;ROUND(NOW(),0)&amp;A19,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A16" s="7">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>19</v>
+    <row r="20" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A20" s="7" t="str">
+        <f>IF(B20&lt;&gt;"",A19+1,"")</f>
+        <v/>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2" t="str">
+        <f ca="1">IF(B20&lt;&gt;"",B20&amp;"_"&amp;ROUND(NOW(),0)&amp;A20,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A17" s="7">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>3</v>
+    <row r="21" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A21" s="7" t="str">
+        <f>IF(B21&lt;&gt;"",A20+1,"")</f>
+        <v/>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2" t="str">
+        <f ca="1">IF(B21&lt;&gt;"",B21&amp;"_"&amp;ROUND(NOW(),0)&amp;A21,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A18" s="7">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>16</v>
+    <row r="22" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A22" s="7" t="str">
+        <f>IF(B22&lt;&gt;"",A21+1,"")</f>
+        <v/>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2" t="str">
+        <f ca="1">IF(B22&lt;&gt;"",B22&amp;"_"&amp;ROUND(NOW(),0)&amp;A22,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A19" s="7">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>4</v>
+    <row r="23" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A23" s="7" t="str">
+        <f>IF(B23&lt;&gt;"",A22+1,"")</f>
+        <v/>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2" t="str">
+        <f ca="1">IF(B23&lt;&gt;"",B23&amp;"_"&amp;ROUND(NOW(),0)&amp;A23,"")</f>
+        <v/>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A20" s="7">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A21" s="7">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="24.75" customHeight="1">
-      <c r="A22" s="7">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>6</v>
+    <row r="24" spans="1:3" ht="24.75" customHeight="1">
+      <c r="A24" s="7" t="str">
+        <f>IF(B24&lt;&gt;"",A23+1,"")</f>
+        <v/>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2" t="str">
+        <f ca="1">IF(B24&lt;&gt;"",B24&amp;"_"&amp;ROUND(NOW(),0)&amp;A24,"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <autoFilter ref="A1:B1" xr:uid="{354B2645-52BC-4BC5-A002-F402E4FA77BA}"/>
-  <conditionalFormatting sqref="B2:B1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+  <conditionalFormatting sqref="B1:B3 B5:B1048576">
+    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4">
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4">
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>